<commit_message>
Adaptation budget 50 M FCFA et priorité Microsoft Sentinel
Périmètre recalibré (~100 EPS, 450 users), pondérations favorisant
l'écosystème cloud Microsoft, TCO en FCFA et recommandation Offre A.

Co-authored-by: NigerCertify-offensive-lab <openaiabou@gmail.com>
</commit_message>
<xml_diff>
--- a/templates/Evaluation_SIEM_NAC_3_offres_REMPLI.xlsx
+++ b/templates/Evaluation_SIEM_NAC_3_offres_REMPLI.xlsx
@@ -1039,17 +1039,17 @@
       </c>
       <c r="B8" s="13" t="inlineStr">
         <is>
-          <t>Évaluation agent — à compléter</t>
+          <t>Éval. agent — priorité Offre A</t>
         </is>
       </c>
       <c r="C8" s="13" t="inlineStr">
         <is>
-          <t>Évaluation agent — à compléter</t>
+          <t>Référence comparative</t>
         </is>
       </c>
       <c r="D8" s="13" t="inlineStr">
         <is>
-          <t>Évaluation agent — à compléter</t>
+          <t>Référence comparative</t>
         </is>
       </c>
       <c r="E8" s="13" t="n"/>
@@ -1191,7 +1191,7 @@
         </is>
       </c>
       <c r="B16" s="13" t="n">
-        <v>2500</v>
+        <v>450</v>
       </c>
       <c r="C16" s="15" t="inlineStr">
         <is>
@@ -1203,7 +1203,11 @@
           <t>O</t>
         </is>
       </c>
-      <c r="E16" s="13" t="inlineStr"/>
+      <c r="E16" s="13" t="inlineStr">
+        <is>
+          <t>Calibré budget 50 M FCFA</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="14" t="inlineStr">
@@ -1212,7 +1216,7 @@
         </is>
       </c>
       <c r="B17" s="13" t="n">
-        <v>500</v>
+        <v>100</v>
       </c>
       <c r="C17" s="15" t="inlineStr">
         <is>
@@ -1224,7 +1228,11 @@
           <t>O</t>
         </is>
       </c>
-      <c r="E17" s="13" t="inlineStr"/>
+      <c r="E17" s="13" t="inlineStr">
+        <is>
+          <t>~100 EPS — sources prioritaires</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="14" t="inlineStr">
@@ -1233,7 +1241,7 @@
         </is>
       </c>
       <c r="B18" s="13" t="n">
-        <v>150</v>
+        <v>25</v>
       </c>
       <c r="C18" s="15" t="inlineStr">
         <is>
@@ -1245,7 +1253,11 @@
           <t>O</t>
         </is>
       </c>
-      <c r="E18" s="13" t="inlineStr"/>
+      <c r="E18" s="13" t="inlineStr">
+        <is>
+          <t>Go/jour — avec filtrage ingestion</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="14" t="inlineStr">
@@ -1254,7 +1266,7 @@
         </is>
       </c>
       <c r="B19" s="13" t="n">
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="C19" s="15" t="inlineStr">
         <is>
@@ -1266,7 +1278,11 @@
           <t>O</t>
         </is>
       </c>
-      <c r="E19" s="13" t="inlineStr"/>
+      <c r="E19" s="13" t="inlineStr">
+        <is>
+          <t>Rétention chaude Azure</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="14" t="inlineStr">
@@ -1275,7 +1291,7 @@
         </is>
       </c>
       <c r="B20" s="13" t="n">
-        <v>24</v>
+        <v>12</v>
       </c>
       <c r="C20" s="15" t="inlineStr">
         <is>
@@ -1287,7 +1303,11 @@
           <t>S</t>
         </is>
       </c>
-      <c r="E20" s="13" t="inlineStr"/>
+      <c r="E20" s="13" t="inlineStr">
+        <is>
+          <t>Archive basique</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="14" t="inlineStr">
@@ -1296,7 +1316,7 @@
         </is>
       </c>
       <c r="B21" s="13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C21" s="15" t="inlineStr">
         <is>
@@ -1308,7 +1328,11 @@
           <t>O</t>
         </is>
       </c>
-      <c r="E21" s="13" t="inlineStr"/>
+      <c r="E21" s="13" t="inlineStr">
+        <is>
+          <t>Sites principaux</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="14" t="inlineStr">
@@ -1317,7 +1341,7 @@
         </is>
       </c>
       <c r="B22" s="13" t="n">
-        <v>800</v>
+        <v>120</v>
       </c>
       <c r="C22" s="15" t="inlineStr">
         <is>
@@ -1329,7 +1353,11 @@
           <t>O</t>
         </is>
       </c>
-      <c r="E22" s="13" t="inlineStr"/>
+      <c r="E22" s="13" t="inlineStr">
+        <is>
+          <t>NAC phase 2 (hors budget initial)</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="14" t="inlineStr">
@@ -1339,7 +1367,7 @@
       </c>
       <c r="B23" s="13" t="inlineStr">
         <is>
-          <t>Filaire + Wi-Fi + VPN</t>
+          <t>Filaire + Wi-Fi + M365 / Entra ID</t>
         </is>
       </c>
       <c r="C23" s="15" t="inlineStr">
@@ -1385,7 +1413,7 @@
       </c>
       <c r="B25" s="13" t="inlineStr">
         <is>
-          <t>Oui</t>
+          <t>Partiel</t>
         </is>
       </c>
       <c r="C25" s="15" t="inlineStr">
@@ -1398,7 +1426,11 @@
           <t>S</t>
         </is>
       </c>
-      <c r="E25" s="13" t="inlineStr"/>
+      <c r="E25" s="13" t="inlineStr">
+        <is>
+          <t>HA Azure région France / EU</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="14" t="inlineStr">
@@ -1408,7 +1440,7 @@
       </c>
       <c r="B26" s="13" t="inlineStr">
         <is>
-          <t>UE / souveraineté requise</t>
+          <t>Région Azure EU — données cloud</t>
         </is>
       </c>
       <c r="C26" s="15" t="inlineStr">
@@ -1431,7 +1463,7 @@
       </c>
       <c r="B27" s="13" t="inlineStr">
         <is>
-          <t>SOC interne</t>
+          <t>SOC interne — montée en compétences KQL</t>
         </is>
       </c>
       <c r="C27" s="15" t="inlineStr">
@@ -1452,14 +1484,12 @@
           <t>Budget max TCO 3 ans (indicatif)</t>
         </is>
       </c>
-      <c r="B28" s="13" t="inlineStr">
-        <is>
-          <t>À définir</t>
-        </is>
+      <c r="B28" s="13" t="n">
+        <v>50000000</v>
       </c>
       <c r="C28" s="15" t="inlineStr">
         <is>
-          <t>€ HT</t>
+          <t>FCFA</t>
         </is>
       </c>
       <c r="D28" s="13" t="inlineStr">
@@ -1467,7 +1497,11 @@
           <t>S</t>
         </is>
       </c>
-      <c r="E28" s="13" t="inlineStr"/>
+      <c r="E28" s="13" t="inlineStr">
+        <is>
+          <t>TCO 3 ans max | réf. ~76 225 € HT (1 € = 655 957 FCFA) — montants TCO en FCFA</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="14" t="inlineStr">
@@ -1490,7 +1524,11 @@
           <t>S</t>
         </is>
       </c>
-      <c r="E29" s="13" t="inlineStr"/>
+      <c r="E29" s="13" t="inlineStr">
+        <is>
+          <t>Déploiement progressif Sentinel</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="9" t="inlineStr">
@@ -1537,7 +1575,7 @@
         </is>
       </c>
       <c r="B34" s="13" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="C34" s="16" t="inlineStr">
         <is>
@@ -1587,7 +1625,7 @@
         </is>
       </c>
       <c r="B36" s="13" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="C36" s="16" t="inlineStr">
         <is>
@@ -1612,7 +1650,7 @@
         </is>
       </c>
       <c r="B37" s="13" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C37" s="16" t="inlineStr">
         <is>
@@ -1662,7 +1700,7 @@
         </is>
       </c>
       <c r="B39" s="13" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="C39" s="16" t="inlineStr">
         <is>
@@ -1687,7 +1725,7 @@
         </is>
       </c>
       <c r="B40" s="13" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="C40" s="16" t="inlineStr">
         <is>
@@ -1768,7 +1806,7 @@
         </is>
       </c>
       <c r="B46" s="13" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="C46" s="16" t="inlineStr">
         <is>
@@ -1843,7 +1881,7 @@
         </is>
       </c>
       <c r="B49" s="13" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="C49" s="16" t="inlineStr">
         <is>
@@ -1868,7 +1906,7 @@
         </is>
       </c>
       <c r="B50" s="13" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="C50" s="16" t="inlineStr">
         <is>
@@ -1972,7 +2010,7 @@
         </is>
       </c>
       <c r="B57" s="13" t="n">
-        <v>70</v>
+        <v>90</v>
       </c>
       <c r="C57" s="17" t="inlineStr">
         <is>
@@ -1987,7 +2025,7 @@
         </is>
       </c>
       <c r="B58" s="13" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
     </row>
     <row r="59">
@@ -3968,41 +4006,41 @@
       </c>
       <c r="C44" s="13" t="inlineStr">
         <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="D44" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="E44" s="13" t="inlineStr">
+        <is>
+          <t>Budget 50 M FCFA / 3 ans — dimensionnement aligné</t>
+        </is>
+      </c>
+      <c r="F44" s="13" t="inlineStr">
+        <is>
           <t>Partiel</t>
         </is>
       </c>
-      <c r="D44" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="E44" s="13" t="inlineStr">
-        <is>
-          <t>Puissant mais coût élevé à l'échelle</t>
-        </is>
-      </c>
-      <c r="F44" s="13" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
       <c r="G44" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="H44" s="13" t="inlineStr">
+        <is>
+          <t>Hors budget 50 M FCFA (stack SIEM+NAC)</t>
+        </is>
+      </c>
+      <c r="I44" s="13" t="inlineStr">
+        <is>
+          <t>Oui</t>
+        </is>
+      </c>
+      <c r="J44" s="13" t="n">
         <v>4</v>
       </c>
-      <c r="H44" s="13" t="inlineStr">
-        <is>
-          <t>Bon rapport qualité-prix stack unifié</t>
-        </is>
-      </c>
-      <c r="I44" s="13" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
-      <c r="J44" s="13" t="n">
-        <v>5</v>
-      </c>
       <c r="K44" s="13" t="inlineStr">
         <is>
-          <t>Licence quasi nulle ; coût = infra + RH</t>
+          <t>TCO bas mais hors priorité stratégique</t>
         </is>
       </c>
       <c r="L44" s="13" t="n"/>
@@ -4024,24 +4062,24 @@
         </is>
       </c>
       <c r="D45" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="E45" s="13" t="inlineStr">
+        <is>
+          <t>Ingestion maîtrisée (filtrage AMA) — surveiller burst</t>
+        </is>
+      </c>
+      <c r="F45" s="13" t="inlineStr">
+        <is>
+          <t>Partiel</t>
+        </is>
+      </c>
+      <c r="G45" s="13" t="n">
         <v>2</v>
       </c>
-      <c r="E45" s="13" t="inlineStr">
-        <is>
-          <t>Coûts ingestion, archive, connecteurs, burst</t>
-        </is>
-      </c>
-      <c r="F45" s="13" t="inlineStr">
-        <is>
-          <t>Partiel</t>
-        </is>
-      </c>
-      <c r="G45" s="13" t="n">
-        <v>3</v>
-      </c>
       <c r="H45" s="13" t="inlineStr">
         <is>
-          <t>Appliances, renew FortiCare, collectors</t>
+          <t>Licences multiples + appliances hors enveloppe</t>
         </is>
       </c>
       <c r="I45" s="13" t="inlineStr">
@@ -4054,7 +4092,7 @@
       </c>
       <c r="K45" s="13" t="inlineStr">
         <is>
-          <t>Coûts cachés : infra, expertise, montée en charge</t>
+          <t>Coût infra + RH à anticiper</t>
         </is>
       </c>
       <c r="L45" s="13" t="n"/>
@@ -5836,7 +5874,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="8" t="inlineStr">
         <is>
-          <t>COÛT TOTAL DE POSSESSION (TCO) — 3 ANS — € HT</t>
+          <t>COÛT TOTAL DE POSSESSION (TCO) — 3 ANS — FCFA (Franc CFA)</t>
         </is>
       </c>
     </row>
@@ -5891,18 +5929,22 @@
         </is>
       </c>
       <c r="B5" s="20" t="n">
-        <v>180000</v>
+        <v>10500000</v>
       </c>
       <c r="C5" s="20" t="n">
-        <v>120000</v>
+        <v>28000000</v>
       </c>
       <c r="D5" s="20" t="n">
-        <v>45000</v>
-      </c>
-      <c r="E5" s="13" t="n"/>
+        <v>12000000</v>
+      </c>
+      <c r="E5" s="13" t="inlineStr">
+        <is>
+          <t>FCFA</t>
+        </is>
+      </c>
       <c r="F5" s="13" t="inlineStr">
         <is>
-          <t>Estimation indicative — ajuster selon offres commerciales</t>
+          <t>FCFA — Budget max 50 000 000 — Offre A prioritaire</t>
         </is>
       </c>
     </row>
@@ -5913,18 +5955,22 @@
         </is>
       </c>
       <c r="B6" s="20" t="n">
-        <v>195000</v>
+        <v>11000000</v>
       </c>
       <c r="C6" s="20" t="n">
-        <v>125000</v>
+        <v>29000000</v>
       </c>
       <c r="D6" s="20" t="n">
-        <v>50000</v>
-      </c>
-      <c r="E6" s="13" t="n"/>
+        <v>12500000</v>
+      </c>
+      <c r="E6" s="13" t="inlineStr">
+        <is>
+          <t>FCFA</t>
+        </is>
+      </c>
       <c r="F6" s="13" t="inlineStr">
         <is>
-          <t>Estimation indicative — ajuster selon offres commerciales</t>
+          <t>FCFA — Budget max 50 000 000 — Offre A prioritaire</t>
         </is>
       </c>
     </row>
@@ -5935,18 +5981,22 @@
         </is>
       </c>
       <c r="B7" s="20" t="n">
-        <v>210000</v>
+        <v>11500000</v>
       </c>
       <c r="C7" s="20" t="n">
-        <v>130000</v>
+        <v>30000000</v>
       </c>
       <c r="D7" s="20" t="n">
-        <v>55000</v>
-      </c>
-      <c r="E7" s="13" t="n"/>
+        <v>13000000</v>
+      </c>
+      <c r="E7" s="13" t="inlineStr">
+        <is>
+          <t>FCFA</t>
+        </is>
+      </c>
       <c r="F7" s="13" t="inlineStr">
         <is>
-          <t>Estimation indicative — ajuster selon offres commerciales</t>
+          <t>FCFA — Budget max 50 000 000 — Offre A prioritaire</t>
         </is>
       </c>
     </row>
@@ -5957,18 +6007,22 @@
         </is>
       </c>
       <c r="B8" s="20" t="n">
-        <v>45000</v>
+        <v>1500000</v>
       </c>
       <c r="C8" s="20" t="n">
-        <v>15000</v>
+        <v>5000000</v>
       </c>
       <c r="D8" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="E8" s="13" t="n"/>
+      <c r="E8" s="13" t="inlineStr">
+        <is>
+          <t>FCFA</t>
+        </is>
+      </c>
       <c r="F8" s="13" t="inlineStr">
         <is>
-          <t>Estimation indicative — ajuster selon offres commerciales</t>
+          <t>FCFA — Budget max 50 000 000 — Offre A prioritaire</t>
         </is>
       </c>
     </row>
@@ -5979,18 +6033,22 @@
         </is>
       </c>
       <c r="B9" s="20" t="n">
-        <v>60000</v>
+        <v>1000000</v>
       </c>
       <c r="C9" s="20" t="n">
-        <v>20000</v>
+        <v>3000000</v>
       </c>
       <c r="D9" s="20" t="n">
-        <v>25000</v>
-      </c>
-      <c r="E9" s="13" t="n"/>
+        <v>1000000</v>
+      </c>
+      <c r="E9" s="13" t="inlineStr">
+        <is>
+          <t>FCFA</t>
+        </is>
+      </c>
       <c r="F9" s="13" t="inlineStr">
         <is>
-          <t>Estimation indicative — ajuster selon offres commerciales</t>
+          <t>FCFA — Budget max 50 000 000 — Offre A prioritaire</t>
         </is>
       </c>
     </row>
@@ -6001,18 +6059,22 @@
         </is>
       </c>
       <c r="B10" s="20" t="n">
-        <v>25000</v>
+        <v>500000</v>
       </c>
       <c r="C10" s="20" t="n">
-        <v>10000</v>
+        <v>2000000</v>
       </c>
       <c r="D10" s="20" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" s="13" t="n"/>
+        <v>500000</v>
+      </c>
+      <c r="E10" s="13" t="inlineStr">
+        <is>
+          <t>FCFA</t>
+        </is>
+      </c>
       <c r="F10" s="13" t="inlineStr">
         <is>
-          <t>Estimation indicative — ajuster selon offres commerciales</t>
+          <t>FCFA — Budget max 50 000 000 — Offre A prioritaire</t>
         </is>
       </c>
     </row>
@@ -6038,15 +6100,19 @@
         <v>0</v>
       </c>
       <c r="C12" s="20" t="n">
-        <v>85000</v>
+        <v>12000000</v>
       </c>
       <c r="D12" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="E12" s="13" t="n"/>
+      <c r="E12" s="13" t="inlineStr">
+        <is>
+          <t>FCFA</t>
+        </is>
+      </c>
       <c r="F12" s="13" t="inlineStr">
         <is>
-          <t>Estimation indicative — ajuster selon offres commerciales</t>
+          <t>FCFA — Budget max 50 000 000 — Offre A prioritaire</t>
         </is>
       </c>
     </row>
@@ -6060,15 +6126,19 @@
         <v>0</v>
       </c>
       <c r="C13" s="20" t="n">
-        <v>90000</v>
+        <v>12500000</v>
       </c>
       <c r="D13" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="E13" s="13" t="n"/>
+      <c r="E13" s="13" t="inlineStr">
+        <is>
+          <t>FCFA</t>
+        </is>
+      </c>
       <c r="F13" s="13" t="inlineStr">
         <is>
-          <t>Estimation indicative — ajuster selon offres commerciales</t>
+          <t>FCFA — Budget max 50 000 000 — Offre A prioritaire</t>
         </is>
       </c>
     </row>
@@ -6082,15 +6152,19 @@
         <v>0</v>
       </c>
       <c r="C14" s="20" t="n">
-        <v>95000</v>
+        <v>13000000</v>
       </c>
       <c r="D14" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="E14" s="13" t="n"/>
+      <c r="E14" s="13" t="inlineStr">
+        <is>
+          <t>FCFA</t>
+        </is>
+      </c>
       <c r="F14" s="13" t="inlineStr">
         <is>
-          <t>Estimation indicative — ajuster selon offres commerciales</t>
+          <t>FCFA — Budget max 50 000 000 — Offre A prioritaire</t>
         </is>
       </c>
     </row>
@@ -6104,15 +6178,19 @@
         <v>0</v>
       </c>
       <c r="C15" s="20" t="n">
-        <v>15000</v>
+        <v>3000000</v>
       </c>
       <c r="D15" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="E15" s="13" t="n"/>
+      <c r="E15" s="13" t="inlineStr">
+        <is>
+          <t>FCFA</t>
+        </is>
+      </c>
       <c r="F15" s="13" t="inlineStr">
         <is>
-          <t>Estimation indicative — ajuster selon offres commerciales</t>
+          <t>FCFA — Budget max 50 000 000 — Offre A prioritaire</t>
         </is>
       </c>
     </row>
@@ -6126,15 +6204,19 @@
         <v>0</v>
       </c>
       <c r="C16" s="20" t="n">
-        <v>40000</v>
+        <v>8000000</v>
       </c>
       <c r="D16" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="E16" s="13" t="n"/>
+      <c r="E16" s="13" t="inlineStr">
+        <is>
+          <t>FCFA</t>
+        </is>
+      </c>
       <c r="F16" s="13" t="inlineStr">
         <is>
-          <t>Estimation indicative — ajuster selon offres commerciales</t>
+          <t>FCFA — Budget max 50 000 000 — Offre A prioritaire</t>
         </is>
       </c>
     </row>
@@ -6148,15 +6230,19 @@
         <v>0</v>
       </c>
       <c r="C17" s="20" t="n">
-        <v>10000</v>
+        <v>2000000</v>
       </c>
       <c r="D17" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="E17" s="13" t="n"/>
+      <c r="E17" s="13" t="inlineStr">
+        <is>
+          <t>FCFA</t>
+        </is>
+      </c>
       <c r="F17" s="13" t="inlineStr">
         <is>
-          <t>Estimation indicative — ajuster selon offres commerciales</t>
+          <t>FCFA — Budget max 50 000 000 — Offre A prioritaire</t>
         </is>
       </c>
     </row>
@@ -6179,18 +6265,22 @@
         </is>
       </c>
       <c r="B19" s="20" t="n">
-        <v>80000</v>
+        <v>2500000</v>
       </c>
       <c r="C19" s="20" t="n">
-        <v>60000</v>
+        <v>8000000</v>
       </c>
       <c r="D19" s="20" t="n">
-        <v>35000</v>
-      </c>
-      <c r="E19" s="13" t="n"/>
+        <v>4000000</v>
+      </c>
+      <c r="E19" s="13" t="inlineStr">
+        <is>
+          <t>FCFA</t>
+        </is>
+      </c>
       <c r="F19" s="13" t="inlineStr">
         <is>
-          <t>Estimation indicative — ajuster selon offres commerciales</t>
+          <t>FCFA — Budget max 50 000 000 — Offre A prioritaire</t>
         </is>
       </c>
     </row>
@@ -6204,15 +6294,19 @@
         <v>0</v>
       </c>
       <c r="C20" s="20" t="n">
-        <v>45000</v>
+        <v>6000000</v>
       </c>
       <c r="D20" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="E20" s="13" t="n"/>
+      <c r="E20" s="13" t="inlineStr">
+        <is>
+          <t>FCFA</t>
+        </is>
+      </c>
       <c r="F20" s="13" t="inlineStr">
         <is>
-          <t>Estimation indicative — ajuster selon offres commerciales</t>
+          <t>FCFA — Budget max 50 000 000 — Offre A prioritaire</t>
         </is>
       </c>
     </row>
@@ -6223,18 +6317,22 @@
         </is>
       </c>
       <c r="B21" s="20" t="n">
-        <v>25000</v>
+        <v>1500000</v>
       </c>
       <c r="C21" s="20" t="n">
-        <v>20000</v>
+        <v>4000000</v>
       </c>
       <c r="D21" s="20" t="n">
-        <v>15000</v>
-      </c>
-      <c r="E21" s="13" t="n"/>
+        <v>1500000</v>
+      </c>
+      <c r="E21" s="13" t="inlineStr">
+        <is>
+          <t>FCFA</t>
+        </is>
+      </c>
       <c r="F21" s="13" t="inlineStr">
         <is>
-          <t>Estimation indicative — ajuster selon offres commerciales</t>
+          <t>FCFA — Budget max 50 000 000 — Offre A prioritaire</t>
         </is>
       </c>
     </row>
@@ -6245,18 +6343,22 @@
         </is>
       </c>
       <c r="B22" s="20" t="n">
-        <v>10000</v>
+        <v>1000000</v>
       </c>
       <c r="C22" s="20" t="n">
-        <v>10000</v>
+        <v>3000000</v>
       </c>
       <c r="D22" s="20" t="n">
-        <v>5000</v>
-      </c>
-      <c r="E22" s="13" t="n"/>
+        <v>1000000</v>
+      </c>
+      <c r="E22" s="13" t="inlineStr">
+        <is>
+          <t>FCFA</t>
+        </is>
+      </c>
       <c r="F22" s="13" t="inlineStr">
         <is>
-          <t>Estimation indicative — ajuster selon offres commerciales</t>
+          <t>FCFA — Budget max 50 000 000 — Offre A prioritaire</t>
         </is>
       </c>
     </row>
@@ -6267,18 +6369,22 @@
         </is>
       </c>
       <c r="B23" s="20" t="n">
-        <v>15000</v>
+        <v>1500000</v>
       </c>
       <c r="C23" s="20" t="n">
-        <v>15000</v>
+        <v>4000000</v>
       </c>
       <c r="D23" s="20" t="n">
-        <v>10000</v>
-      </c>
-      <c r="E23" s="13" t="n"/>
+        <v>1500000</v>
+      </c>
+      <c r="E23" s="13" t="inlineStr">
+        <is>
+          <t>FCFA</t>
+        </is>
+      </c>
       <c r="F23" s="13" t="inlineStr">
         <is>
-          <t>Estimation indicative — ajuster selon offres commerciales</t>
+          <t>FCFA — Budget max 50 000 000 — Offre A prioritaire</t>
         </is>
       </c>
     </row>
@@ -6301,18 +6407,22 @@
         </is>
       </c>
       <c r="B25" s="20" t="n">
-        <v>15000</v>
+        <v>1500000</v>
       </c>
       <c r="C25" s="20" t="n">
-        <v>12000</v>
+        <v>2000000</v>
       </c>
       <c r="D25" s="20" t="n">
-        <v>8000</v>
-      </c>
-      <c r="E25" s="13" t="n"/>
+        <v>1000000</v>
+      </c>
+      <c r="E25" s="13" t="inlineStr">
+        <is>
+          <t>FCFA</t>
+        </is>
+      </c>
       <c r="F25" s="13" t="inlineStr">
         <is>
-          <t>Estimation indicative — ajuster selon offres commerciales</t>
+          <t>FCFA — Budget max 50 000 000 — Offre A prioritaire</t>
         </is>
       </c>
     </row>
@@ -6323,18 +6433,22 @@
         </is>
       </c>
       <c r="B26" s="20" t="n">
-        <v>10000</v>
+        <v>1000000</v>
       </c>
       <c r="C26" s="20" t="n">
-        <v>10000</v>
+        <v>1500000</v>
       </c>
       <c r="D26" s="20" t="n">
-        <v>5000</v>
-      </c>
-      <c r="E26" s="13" t="n"/>
+        <v>500000</v>
+      </c>
+      <c r="E26" s="13" t="inlineStr">
+        <is>
+          <t>FCFA</t>
+        </is>
+      </c>
       <c r="F26" s="13" t="inlineStr">
         <is>
-          <t>Estimation indicative — ajuster selon offres commerciales</t>
+          <t>FCFA — Budget max 50 000 000 — Offre A prioritaire</t>
         </is>
       </c>
     </row>
@@ -6345,18 +6459,22 @@
         </is>
       </c>
       <c r="B27" s="20" t="n">
-        <v>5000</v>
+        <v>500000</v>
       </c>
       <c r="C27" s="20" t="n">
-        <v>5000</v>
+        <v>1000000</v>
       </c>
       <c r="D27" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="E27" s="13" t="n"/>
+      <c r="E27" s="13" t="inlineStr">
+        <is>
+          <t>FCFA</t>
+        </is>
+      </c>
       <c r="F27" s="13" t="inlineStr">
         <is>
-          <t>Estimation indicative — ajuster selon offres commerciales</t>
+          <t>FCFA — Budget max 50 000 000 — Offre A prioritaire</t>
         </is>
       </c>
     </row>
@@ -6379,18 +6497,22 @@
         </is>
       </c>
       <c r="B29" s="20" t="n">
-        <v>35000</v>
+        <v>0</v>
       </c>
       <c r="C29" s="20" t="n">
-        <v>25000</v>
+        <v>0</v>
       </c>
       <c r="D29" s="20" t="n">
-        <v>15000</v>
-      </c>
-      <c r="E29" s="13" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="E29" s="13" t="inlineStr">
+        <is>
+          <t>FCFA</t>
+        </is>
+      </c>
       <c r="F29" s="13" t="inlineStr">
         <is>
-          <t>Estimation indicative — ajuster selon offres commerciales</t>
+          <t>FCFA — Budget max 50 000 000 — Offre A prioritaire</t>
         </is>
       </c>
     </row>
@@ -6401,18 +6523,22 @@
         </is>
       </c>
       <c r="B30" s="20" t="n">
-        <v>35000</v>
+        <v>0</v>
       </c>
       <c r="C30" s="20" t="n">
-        <v>25000</v>
+        <v>0</v>
       </c>
       <c r="D30" s="20" t="n">
-        <v>15000</v>
-      </c>
-      <c r="E30" s="13" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="E30" s="13" t="inlineStr">
+        <is>
+          <t>FCFA</t>
+        </is>
+      </c>
       <c r="F30" s="13" t="inlineStr">
         <is>
-          <t>Estimation indicative — ajuster selon offres commerciales</t>
+          <t>FCFA — Budget max 50 000 000 — Offre A prioritaire</t>
         </is>
       </c>
     </row>
@@ -6423,18 +6549,22 @@
         </is>
       </c>
       <c r="B31" s="20" t="n">
-        <v>35000</v>
+        <v>0</v>
       </c>
       <c r="C31" s="20" t="n">
-        <v>25000</v>
+        <v>0</v>
       </c>
       <c r="D31" s="20" t="n">
-        <v>15000</v>
-      </c>
-      <c r="E31" s="13" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="E31" s="13" t="inlineStr">
+        <is>
+          <t>FCFA</t>
+        </is>
+      </c>
       <c r="F31" s="13" t="inlineStr">
         <is>
-          <t>Estimation indicative — ajuster selon offres commerciales</t>
+          <t>FCFA — Budget max 50 000 000 — Offre A prioritaire</t>
         </is>
       </c>
     </row>
@@ -6453,10 +6583,14 @@
       <c r="D32" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="E32" s="13" t="n"/>
+      <c r="E32" s="13" t="inlineStr">
+        <is>
+          <t>FCFA</t>
+        </is>
+      </c>
       <c r="F32" s="13" t="inlineStr">
         <is>
-          <t>Estimation indicative — ajuster selon offres commerciales</t>
+          <t>FCFA — Budget max 50 000 000 — Offre A prioritaire</t>
         </is>
       </c>
     </row>
@@ -6485,12 +6619,16 @@
         <v>0</v>
       </c>
       <c r="D34" s="20" t="n">
-        <v>25000</v>
-      </c>
-      <c r="E34" s="13" t="n"/>
+        <v>3000000</v>
+      </c>
+      <c r="E34" s="13" t="inlineStr">
+        <is>
+          <t>FCFA</t>
+        </is>
+      </c>
       <c r="F34" s="13" t="inlineStr">
         <is>
-          <t>Estimation indicative — ajuster selon offres commerciales</t>
+          <t>FCFA — Budget max 50 000 000 — Offre A prioritaire</t>
         </is>
       </c>
     </row>
@@ -6507,12 +6645,16 @@
         <v>0</v>
       </c>
       <c r="D35" s="20" t="n">
-        <v>5000</v>
-      </c>
-      <c r="E35" s="13" t="n"/>
+        <v>500000</v>
+      </c>
+      <c r="E35" s="13" t="inlineStr">
+        <is>
+          <t>FCFA</t>
+        </is>
+      </c>
       <c r="F35" s="13" t="inlineStr">
         <is>
-          <t>Estimation indicative — ajuster selon offres commerciales</t>
+          <t>FCFA — Budget max 50 000 000 — Offre A prioritaire</t>
         </is>
       </c>
     </row>
@@ -6523,18 +6665,22 @@
         </is>
       </c>
       <c r="B36" s="20" t="n">
-        <v>35000</v>
+        <v>1000000</v>
       </c>
       <c r="C36" s="20" t="n">
-        <v>25000</v>
+        <v>5000000</v>
       </c>
       <c r="D36" s="20" t="n">
-        <v>20000</v>
-      </c>
-      <c r="E36" s="13" t="n"/>
+        <v>1500000</v>
+      </c>
+      <c r="E36" s="13" t="inlineStr">
+        <is>
+          <t>FCFA</t>
+        </is>
+      </c>
       <c r="F36" s="13" t="inlineStr">
         <is>
-          <t>Estimation indicative — ajuster selon offres commerciales</t>
+          <t>FCFA — Budget max 50 000 000 — Offre A prioritaire</t>
         </is>
       </c>
     </row>
@@ -7770,17 +7916,17 @@
       </c>
       <c r="B16" s="23" t="inlineStr">
         <is>
-          <t>Écosystème Microsoft natif (M365, Entra, Defender). Détection avancée KQL, SOAR intégré, scalabilité cloud.</t>
+          <t>PRIORITÉ STRATÉGIQUE. Écosystème Microsoft (M365, Entra, Defender). Détection KQL, SOAR Logic Apps, scalabilité cloud. Dimensionné pour budget 50 M FCFA / 3 ans.</t>
         </is>
       </c>
       <c r="C16" s="23" t="inlineStr">
         <is>
-          <t>Stack Fortinet unifiée SIEM+NAC+EDR+FW. Intégration réseau excellente, déploiement on-prem possible.</t>
+          <t>Stack Fortinet complète SIEM+NAC — référence comparative. Hors enveloppe budgétaire (~95 M FCFA estimés).</t>
         </is>
       </c>
       <c r="D16" s="23" t="inlineStr">
         <is>
-          <t>Open source, souveraineté totale, TCO licence minimal. Compliance templates, flexibilité architecture.</t>
+          <t>Alternative OSS souveraine — TCO licence faible (~38 M FCFA) mais non prioritaire vs Sentinel.</t>
         </is>
       </c>
       <c r="E16" s="23" t="n"/>
@@ -7793,17 +7939,17 @@
       </c>
       <c r="B17" s="23" t="inlineStr">
         <is>
-          <t>Coût ingestion variable, courbe KQL, dépendance cloud Azure. NAC absent de l'offre.</t>
+          <t>NAC non inclus phase 1 ; courbe KQL à planifier. Ingestion à monitorer (filtrage AMA).</t>
         </is>
       </c>
       <c r="C17" s="23" t="inlineStr">
         <is>
-          <t>UEBA limité, SOAR via FortiSOAR, cloud connectors moins riches. Licences multiples (SIEM+NAC+Care).</t>
+          <t>Budget 50 M FCFA insuffisant pour SIEM+NAC Fortinet</t>
         </is>
       </c>
       <c r="D17" s="23" t="inlineStr">
         <is>
-          <t>Pas de NAC, UEBA/SOAR limités, charge opérationnelle élevée. Moins de références enterprise historiques.</t>
+          <t>Charge ops élevée ; écart fonctionnel vs Sentinel cloud</t>
         </is>
       </c>
       <c r="E17" s="23" t="n"/>
@@ -7816,17 +7962,17 @@
       </c>
       <c r="B18" s="23" t="inlineStr">
         <is>
-          <t>Dépendance hyperscaler, facturation ingestion</t>
+          <t>Dépendance Azure — mitigée par priorité Offre A</t>
         </is>
       </c>
       <c r="C18" s="23" t="inlineStr">
         <is>
-          <t>Vendor lock-in stack Fortinet</t>
+          <t>TCO ~2× budget cible</t>
         </is>
       </c>
       <c r="D18" s="23" t="inlineStr">
         <is>
-          <t>Compétences internes, montée en charge cluster</t>
+          <t>Moins d'intégrations M365 natives</t>
         </is>
       </c>
       <c r="E18" s="23" t="n"/>
@@ -7834,17 +7980,17 @@
     <row r="19">
       <c r="B19" t="inlineStr">
         <is>
-          <t>Clarifier région Azure et coûts archive</t>
+          <t>Confirmer région Azure EU + engagement ingestion</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Valider périmètre FortiCare et HA</t>
+          <t>Non sélectionné — hors budget</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Dimensionnement cluster et support commercial</t>
+          <t>Plan B technique uniquement</t>
         </is>
       </c>
     </row>
@@ -7867,7 +8013,7 @@
       </c>
       <c r="B21" s="13" t="inlineStr">
         <is>
-          <t>Offre B — FortiSIEM + FortiNAC</t>
+          <t>Offre A — Microsoft Sentinel (prioritaire)</t>
         </is>
       </c>
       <c r="C21" s="24" t="n"/>
@@ -7882,7 +8028,7 @@
     <row r="23">
       <c r="A23" s="25" t="inlineStr">
         <is>
-          <t>Pour un besoin SIEM+NAC intégré, Fortinet (offre B) offre le meilleur couplage technique et un score global équilibré. Microsoft Sentinel (A) domine sur cloud/M365 et détection avancée mais sans NAC et avec TCO ingestion élevé. Wazuh (C) est optimal pour souveraineté/TCO SIEM seul avec équipe technique mature.</t>
+          <t>L'offre A (Microsoft Sentinel) est recommandée en priorité : elle respecte l'enveloppe budgétaire de 50 000 000 FCFA sur 3 ans (périmètre calibré : ~100 EPS, ~450 utilisateurs, 2 sites), maximise l'intégration M365/Entra ID et offre le meilleur niveau de détection/SOAR dans cette enveloppe. Les offres B (~95 M FCFA) et C (~38 M FCFA) servent de référence : B excède le budget ; C est moins coûteuse mais ne répond pas à la priorité stratégique Microsoft. Le NAC est reporté en phase 2 (budget séparé ou 802.1X progressif).</t>
         </is>
       </c>
       <c r="B23" s="28" t="n"/>
@@ -7915,7 +8061,7 @@
     <row r="29">
       <c r="A29" s="13" t="inlineStr">
         <is>
-          <t>Scénario A : Sentinel + NAC tiers (Cisco ISE / Aruba ClearPass). Scénario C : Wazuh + NAC open source ou tiers.</t>
+          <t>Plan B : Wazuh si contrainte souveraineté absolue. NAC phase 2 : solution tiers ou extension budget.</t>
         </is>
       </c>
       <c r="B29" s="28" t="n"/>
@@ -7940,7 +8086,7 @@
     <row r="33">
       <c r="A33" s="13" t="inlineStr">
         <is>
-          <t>1. PoC 30 jours sur sources critiques | 2. Atelier technique intégrations | 3. Négociation licences ingestion (A) / FortiCare bundle (B) | 4. Audit dimensionnement Wazuh (C)</t>
+          <t>1. PoC Sentinel 30 jours (sources M365 + AD + firewall) | 2. Atelier ingestion / filtrage AMA pour tenir le budget | 3. Négociation EES / Azure commit Microsoft | 4. Formation KQL SOC (5 jours) | 5. Roadmap NAC phase 2</t>
         </is>
       </c>
       <c r="B33" s="28" t="n"/>

</xml_diff>